<commit_message>
Add MIRAconnect portal checks to MIRA 604 register
New "Portal checks" sheet (P001-P032) records the validations the
MIRAconnect 604 filing page applies: the 10 server errors returned by
Check and Calculate, browser-side checks on submit, and the required
columns on each table row, each mapped to the PDF box and Rule register
ID. Read me gains a "Portal vs PDF" summary.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mira-604/MIRA_604_v26.1_validation_register.xlsx
+++ b/mira-604/MIRA_604_v26.1_validation_register.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates &amp; thresholds" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field inventory" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portal checks" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -258,6 +259,25 @@
     <tableColumn id="11" name="Has event script"/>
     <tableColumn id="12" name="Format test"/>
     <tableColumn id="13" name="Dropdown items"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PortalChecks" displayName="PortalChecks" ref="A1:J33" headerRowCount="1">
+  <autoFilter ref="A1:J33"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="ID"/>
+    <tableColumn id="2" name="Portal screen/step"/>
+    <tableColumn id="3" name="Field"/>
+    <tableColumn id="4" name="Matching PDF section/box"/>
+    <tableColumn id="5" name="Required in portal"/>
+    <tableColumn id="6" name="Format/limit"/>
+    <tableColumn id="7" name="Exact error message"/>
+    <tableColumn id="8" name="How found"/>
+    <tableColumn id="9" name="PDF rule (from Rule register)"/>
+    <tableColumn id="10" name="Difference"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -552,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -562,228 +582,312 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MIRA 604 Income Tax Return – Validation Register</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
+          <t xml:space="preserve">MIRA 604 Income Tax Return - Validation Register</t>
+        </is>
+      </c>
+      <c r="B1" s="2"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Form version</t>
+          <t xml:space="preserve">Form version</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>26.1 (fillable PDF supplied 19 Oct 2026; built in Adobe LiveCycle Designer ES 9.0, XFA)</t>
+          <t xml:space="preserve">26.1 (fillable PDF supplied 19 Oct 2026; built in Adobe LiveCycle Designer ES 9.0, XFA)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t xml:space="preserve">Source</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Extracted directly from the form's embedded XFA template (field settings, calculation scripts, event scripts, validation scripts), cross-checked against the printed instructions on all 17 pages.</t>
+          <t xml:space="preserve">Extracted directly from the form's embedded XFA template (field settings, calculation scripts, event scripts, validation scripts), cross-checked against the printed instructions on all 17 pages.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t xml:space="preserve">Scope</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Rules built into the PDF only. MIRAconnect applies its own checks at submission; those are not in this file.</t>
+          <t xml:space="preserve">Rules built into the PDF, plus the checks MIRAconnect applies on its own 604 filing page (see 'Portal checks' and 'Portal vs PDF' below).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="n"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Key findings</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n"/>
+          <t xml:space="preserve">Key findings</t>
+        </is>
+      </c>
+      <c r="B6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>There are NO mandatory-field checks. Any box can be left empty.</t>
+          <t xml:space="preserve">There are NO mandatory-field checks. Any box can be left empty.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Only one hard error message exists: donation dates must be DDMMYYYY (page 15).</t>
+          <t xml:space="preserve">Only one hard error message exists: donation dates must be DDMMYYYY (page 15).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Most 'validation' is done by locking: ~150 boxes are auto-calculated and read-only, and ~35 boxes open or lock depending on taxpayer type, residency, PE, shipping, cash basis, Section VIII and Box 204.</t>
+          <t xml:space="preserve">Most 'validation' is done by locking: ~150 boxes are auto-calculated and read-only, and ~35 boxes open or lock depending on taxpayer type, residency, PE, shipping, cash basis, Section VIII and Box 204.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="A10" s="8211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Note 1–3 allocation rules (Zakat, sponsorship, donations) and the 5% donation cap are fully automated.</t>
+          <t xml:space="preserve">Note 1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Statements of capital allowance and balancing allowance/charge have NO row-level calculations: only the column totals are summed.</t>
+          <t xml:space="preserve">Statements of capital allowance and balancing allowance/charge have NO row-level calculations: only the column totals are summed.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>14 defects, quirks or gaps found in the scripts. See the 'Defects' sheet. Most important: individual tax brackets break for accounting periods crossing a calendar year end, and Section VIII = Yes does not clear several boxes.</t>
+          <t xml:space="preserve">14 defects, quirks or gaps found in the scripts. See the 'Defects' sheet. Most important: individual tax brackets break for accounting periods crossing a calendar year end, and Section VIII = Yes does not clear several boxes.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Scripts only run in Adobe Acrobat/Reader. Other PDF viewers show a flat form with no calculations.</t>
+          <t xml:space="preserve">Scripts only run in Adobe Acrobat/Reader. Other PDF viewers show a flat form with no calculations.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="n"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Sheets</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n"/>
+          <t xml:space="preserve">Sheets</t>
+        </is>
+      </c>
+      <c r="B15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Rule register</t>
+          <t xml:space="preserve">Rule register</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>One row per rule: page, section, box, XFA field, rule type, what the form does, printed instruction, whether the form enforces it, observation.</t>
+          <t xml:space="preserve">One row per rule: page, section, box, XFA field, rule type, what the form does, printed instruction, whether the form enforces it, observation.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Conditional locks</t>
+          <t xml:space="preserve">Conditional locks</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Which answer opens or locks which boxes.</t>
+          <t xml:space="preserve">Which answer opens or locks which boxes.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Rates &amp; thresholds</t>
+          <t xml:space="preserve">Rates &amp; thresholds</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Every hard-coded number in the scripts.</t>
+          <t xml:space="preserve">Every hard-coded number in the scripts.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Defects</t>
+          <t xml:space="preserve">Defects</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Script behaviour that differs from the printed form or is likely wrong.</t>
+          <t xml:space="preserve">Script behaviour that differs from the printed form or is likely wrong.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Field inventory</t>
+          <t xml:space="preserve">Field inventory</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>All 672 fields with their technical limits (type, comb cells, max characters, picture, read-only, calculated).</t>
+          <t xml:space="preserve">All 672 fields with their technical limits (type, comb cells, max characters, picture, read-only, calculated).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-      <c r="B21" s="2" t="n"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal checks</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Checks MIRAconnect applies to the 604 return (server errors from 'Check and Calculate', browser checks, table-row rules), mapped to the PDF box and Rule register ID.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Enforced? legend</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Yes = the form forces it (calculation, lock or error). Partly = format/limit only. No = printed instruction only, not checked.</t>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enforced? legend</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes = the form forces it (calculation, lock or error). Partly = format/limit only. No = printed instruction only, not checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal vs PDF</t>
+        </is>
+      </c>
+      <c r="B25" s="2"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How found</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIRAconnect 604 filing page for tax year 2025 (form shown as MIRA 604 Version 26.1), 20 Oct 2026. The page code was read, and 'Check and Calculate' was pressed once on an existing draft with no fields changed. Nothing was saved, submitted or paid. Taxpayer names, TINs and bank details are not recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandatory only in portal (server)</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate refused the return with 10 errors: II-b functional currency, preceding year (a-d) and this year (e-h); III presentation currency; XIII at least one bank account; upload of directors report, audit report and financial statements; declaration contact number; Schedule 4 items 4.3(a) and 4.3(b) (a loan row or the no-loans tick). None of these is required in the PDF (R031).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandatory only in portal (browser)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 item 3A cannot be blank (enter 0). Submit stays disabled until the offence-warning box is ticked. Each table row (bank accounts, immovable property, financial interest, group companies, beneficial owners, donations, Schedule 4 and 6 tables) has required columns and cannot be saved half-filled; beneficial owners need ownership OR controlling interest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conflicts with the PDF</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Donation date: PDF is DDMMYYYY text with its own error and 30/50-character limits on donee/details; portal uses a date picker with no length limits. Group company TIN: PDF numeric 7 cells; portal free text, unchecked. Financial interest %: portal 0-100, PDF unchecked. Property investment: portal must be &gt; 0, PDF unchecked. Beneficial owners: PDF one row; portal many rows, all required. Schedules 4-6 and the sponsorship statements exist in the portal but are not in the PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server rules this return already passes only show when broken, so they are not listed: e.g. declaration name/designation, accounting period, audit opinion, box caps and Schedule 1 links, residency and taxpayer-type conditions. Also untested: what triggers the bank-account and upload requirements (e.g. individuals, 'Not required to audit'), server-side errors when saving table rows, the s.11(r) confirmation, and the Submit step itself (not pressed).</t>
         </is>
       </c>
     </row>
@@ -37404,4 +37508,1749 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal screen/step</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Field</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matching PDF section/box</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Required in portal</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Format/limit</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact error message</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How found</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF rule (from Rule register)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 item 4.3(a) Loans from associates</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1 (Schedule 4 is portal-only)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: when Schedule 4 applies. Add at least one loan row, or tick 'did not receive any loans from associates' (A_SCH4_NO_LOANS_FROM_ASS_Checked).</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grid row; tick box zeroes the requirement</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You must fill all boxes 4.3 (a) in Schedule 4</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only mandatory item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 item 4.3(b) Loans to associates</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1 (Schedule 4 is portal-only)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: when Schedule 4 applies. Add at least one loan row, or tick 'did not give any loans to associates' (A_SCH4_NO_LOANS_TO_ASS_Checked).</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grid row; tick box zeroes the requirement</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You must fill all boxes 4.3 (b) in Schedule 4</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only mandatory item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">II-b Functional currency, preceding tax year, options (a)-(d)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">II-b Functional currency (other years)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes (fired on a non-first-year return)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single choice (a)-(d)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item (II-b) cannot be left blank. Please select check box (a), (b), (c) or (d).</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R037</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: radio, not checked, can be blank. Portal: mandatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">II-b Functional currency, this tax year, options (e)-(h)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">II-b Functional currency (other years)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: if this is not the first tax year</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single choice (e)-(h)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item (II-b) cannot be left blank if this is not your first tax year. Please select check box (e), (f), (g) or (h).</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R037</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: not checked. Portal: mandatory for non-first years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">III Presentation currency</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">III Presentation currency</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single choice: Rufiyaa / United States Dollar</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please select the presentation currency</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R039</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: radio, can be blank. Portal: mandatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIII Bank accounts (at least one row)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIII Bank accounts</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes (observed for this return; exemptions, e.g. by taxpayer type, not visible)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At least one row in the bank account table</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item XIII on page 3 cannot be left blank. Please enter the details of bank accounts as required.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R050</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: free-text row, not checked. Portal: at least one bank account required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supporting documents: Directors' report upload</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document checklist (Directors' report)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional (fired for this return; trigger not visible in page code, likely taxpayer type / audit opinion)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF upload, document type 'Directors' Report'</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please upload directors report</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R032</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: a tick box only, not checked. Portal: the file must be uploaded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supporting documents: Auditor's report upload</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document checklist (Audit report); IV Audit opinion</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional (fired for this return; trigger not visible, likely audit opinion other than 'Not required to audit')</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF upload, document type 'Auditor's Report'; declaration tick that the report is for this tax year</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please upload audit report</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R032, R040</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: tick box only, no link to audit opinion. Portal: upload required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supporting documents: financial statements</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document checklist (P&amp;L, financial position, cash flows, changes in equity, notes)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional (fired for this return)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF upload as 'Other Supporting Documents'</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please upload statement of comprehensive income, statement of cash flows, notes to the financial statements, statement of financial position and statement of changes in equity as other supporting documents</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R032</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: tick boxes only. Portal: the files must be uploaded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: Person to contact, contact number</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: Contact Number</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Format not visible in page code</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please enter contact number</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (Check and Calculate, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R028</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: numeric only, not required. Portal: mandatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate / Submit (browser, before sending)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 item 3A (A_SCH4_All_ASSOS_IR and A_SCH4_All_ASSOS_EP)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: when Schedule 4 is showing</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Must not be blank; enter 0 if nothing to report (blank field outlined red)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item no 3A cannot be left blank; if there is no sale/purchase to report, then enter 0.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (mainPostBtn click handler)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only. A browser alert stops the form being sent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whole form (browser)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When Schedule 4 is shown</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section A boxes 1-5, 9 vs 11, 12, 14, 17, 18, 21, 51</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule: hidden only if just remuneration boxes (1-5, 9) have values and boxes 11, 12, 14, 17, 18, 21, 51 are all empty; shown otherwise (including all Section B filers)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Display rule</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (toggleSchedule4)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decides when P001, P002, P011 apply. Not in PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Submit (browser)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Offence-warning acknowledgement in the Submit pop-up</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration / IMPORTANT notice</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes: Submit stays disabled until ticked</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tick box (HasAcknowledgedTaxDeclarationOffenceWarning)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no message; button disabled)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (submitConfirmationModal)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only step. Not tested (Submit not pressed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header / Section VIII (browser)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non-resident shipping/aircraft operator: 'did not derive s.11(r) income' confirmation</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIII Section 11(r) only?; Boxes 204-215</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: non-resident shipping/aircraft operator (entity type 5)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tick box A_NO_S11R_INC_CONFIRM_Checked mirrored in a pop-up</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are a non-resident shipping/aircraft operator. Please indicate in the Box below that you did not derive any income as specified in s.11(r) of the Income Tax Act. If you did derive such income, you must complete Boxes 204 to 215</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (nonResShipConfirmModal)</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R045</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal adds an explicit confirmation. Whether the server enforces it was not tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section A / B deductions (browser)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box 27 / Box 155 Donations</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boxes 27, 155</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not typed: filled from the Statement of Donations table</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Typing resets the box to 0 and opens the donations table</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This value will be auto populated from statement of donations table. Please scroll down and fill the statement of donations table.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (A_A_DED_DONATIONS input handler)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R072, R133</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same intent as the PDF (locked, filled from the donations total).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIII Bank accounts table (row save)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account name, Account number, Currency, Name and address of bank including the country</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIII Bank accounts</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes, all 4 fields, for each row</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Free text; Currency is a dropdown (MIRA currency list)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Account name field is required. / The Account number field is required. / The Currency field is required. / The Name and address of bank including the country field is required.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R050</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: no required fields. Portal: an incomplete row cannot be saved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XII Immovable property table (row save)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name/address/location, Purpose, Country, Total investment (at cost)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XII Immovable property</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes, all 4 fields</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Country dropdown; investment numeric, minimum 1</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Name, address and location of the property field is required. / The Purpose for which the property is used (eg. Rental property) field is required. / The Country field is required. / The Total investment (at cost) field is required. / Total investment (at cost) must be greater than 0</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R049</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: no checks. Portal: required, and investment must be &gt; 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XI Financial interest table (row save)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Country of incorporation, Currency, Investment, Percentage</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XI Shares/interest outside Maldives</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Country and Currency required; Name, Investment, Percentage optional</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investment numeric; Percentage 0-100</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Country of incorporation field is required. / The Currency field is required. / The field Percentage of total investment must be between 0 and 100.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R048</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: no range on %. Portal: 0-100 and required country/currency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X Group companies table (row save)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Country of residence (Name and TIN optional)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X Group companies</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Country required</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TIN is free text with no format check; Country dropdown</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Country of residence field is required.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R047</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conflict: PDF TIN is numeric 7 cells; portal TIN is unchecked free text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIV Beneficial owners table (row save)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name, Date of birth, Nationality, National ID/Passport, Nature of ownership / controlling interest</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIV Beneficial owners</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name, DOB, Nationality, ID required; ownership OR controlling interest required</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DOB date, cannot be after today; dropdowns for nationality and both interest types</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Name field is required. / The Date of birth field is required. / The Nationality field is required. / The National ID/Passport number field is required. / Nature of ownership interest or nature of controlling interest is required. / Nature of ownership interest or nature of controlling interest is required. Both cannot be left blank.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val, onBeneficialOwnerEdit)</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R051</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: one row, nothing required. Portal: unlimited rows, each fully required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statement of donations table (row save)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No., Date, Name of donee, Details, Amount</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Donations (page 15)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes, all 5 fields</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No. at least 1; date picker; amount numeric, not negative; no length limits seen</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The No. field is required. / Number should ge greater than or equal to 1 / The Date of donation field is required. / The Name of donee field is required. / The Details of donation field is required. / The Amount of donation field is required. / Donation amount cannot be negative</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R177, R178, R179</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conflict: PDF date is DDMMYYYY text with a format error and 30/50-char limits; portal uses a date picker and has no length limits. Neither checks the date is in the tax year (client side).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statements of sponsorship (teams / media)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All columns</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note 2 boxes 34-36 / 162-164</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No client-side required fields</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printed note: payment date must fall within the tax year</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none found)</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date-in-year rule is printed only; any server check not tested. Not in PDF register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 tables (row save)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shareholders, own shares, ultimate holding company</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Country of residence required</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Percentage and tax rate numeric, not negative</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Country of residence field is required. / Percentage of shareholding cannot be negative / Tax rate cannot be negative</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 Branches table (row save)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name, Location/Country, Percentage, Tax rate</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes, all 4 fields</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Numeric, not negative</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Name field is required. / The Location / Country field is required. / The Percentage of shareholding field is required. / The Tax rate field is required.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 Beneficial owner table (row save)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name, Country of residence, Identification number</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes, all 3 fields</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Country dropdown</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Name field is required. / The Country of residence field is required. / The Identification number field is required.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 Sales to / purchases from associates (row save)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfer pricing method; (purchases) Tax rate, Amount</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP method required in both; tax rate and amount required for purchases</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dropdown of TP methods; amounts and rates not negative</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Transfer pricing method* field is required. / The Tax rate field is required. / The Amount field is required. / Amount cannot be negative / Tax rate cannot be negative</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only. Sales and purchases tables are not symmetric (sales: amount and rate optional).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 Loans from / to associates (row save)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effective year</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effective year required</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date; loan value, rate, interest, balances numeric (no sign check)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Effective year field is required.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (grid editor data-val)</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 'none of these' tick boxes</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rent/royalty, Services, Financial, Others groups</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lock, not a requirement</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ticking sets the group's boxes to 0.00 and locks them</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (bindCheckToggle)</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only lock logic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 6 beneficial owner tables (row save)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same columns as XIV</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As P020</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As P020</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same messages as P020</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (onSch6BeneficialOwnerEdit)</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 6 items 9-13</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share / interest / option / IP fields</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lock: items open only when the matching item 8 ticks are set (8.2/8.5; 8.3/8.4/8.6/8.7; 8.8; 8.10/8.11/8.14; 8.12/8.13/8.15)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unticking clears the values</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (toggleItem9-13)</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only lock logic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whole form (browser)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All 634 amount boxes</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All numeric boxes</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No (format only)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Must be a number; commas are stripped on focus</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The field &lt;box&gt; must be a number.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (data-val-number)</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Field inventory</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same intent as the PDF numeric pictures; portal has no fixed digit limits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whole form (browser)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accounting period From / To, Declaration date, Schedule 6 disposal date</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header accounting period; Declaration date</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Format only (received date also flagged required but is pre-filled)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Must be a valid date</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The field A_PERIOD_FROM must be a date. (same pattern for A_PERIOD_TO, A_DEC_DATE, A_SCH6_DISPOSE_DATE)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code (data-val-date)</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R012, R029</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF uses DDMMYYYY comb cells; neither checks To is after From (client side).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add portal test script sheet to MIRA 604 register
New "Portal test script" sheet (T00-T37) lists Check and Calculate
tests, ordered by materiality, to surface server-side rules that only
appear when broken: what to change, expected result, known message,
restore step and links to Portal checks / Rule register. Actual message
and Outcome columns are left for the tester. Read me explains how to
run it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mira-604/MIRA_604_v26.1_validation_register.xlsx
+++ b/mira-604/MIRA_604_v26.1_validation_register.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field inventory" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portal checks" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portal test script" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -278,6 +279,26 @@
     <tableColumn id="8" name="How found"/>
     <tableColumn id="9" name="PDF rule (from Rule register)"/>
     <tableColumn id="10" name="Difference"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="PortalTests" displayName="PortalTests" ref="A1:K39" headerRowCount="1">
+  <autoFilter ref="A1:K39"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="Test ID"/>
+    <tableColumn id="2" name="Priority"/>
+    <tableColumn id="3" name="Area / PDF box"/>
+    <tableColumn id="4" name="Starting state"/>
+    <tableColumn id="5" name="Change to make"/>
+    <tableColumn id="6" name="Expected result"/>
+    <tableColumn id="7" name="Known message"/>
+    <tableColumn id="8" name="Actual message (fill in)"/>
+    <tableColumn id="9" name="Outcome (fill in)"/>
+    <tableColumn id="10" name="Restore after test"/>
+    <tableColumn id="11" name="Links (Portal checks / Rule register)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -572,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -888,6 +909,54 @@
       <c r="B30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Server rules this return already passes only show when broken, so they are not listed: e.g. declaration name/designation, accounting period, audit opinion, box caps and Schedule 1 links, residency and taxpayer-type conditions. Also untested: what triggers the bank-account and upload requirements (e.g. individuals, 'Not required to audit'), server-side errors when saving table rows, the s.11(r) confirmation, and the Submit step itself (not pressed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal test script</t>
+        </is>
+      </c>
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Purpose</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Step-by-step Check and Calculate tests (sheet 'Portal test script', T00-T37) to find the server rules that only appear when broken. Ordered High &gt; Medium &gt; Low by how likely each is to block a filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How to run</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run T00-T02 first. Change ONE thing per test, press Check and Calculate only (never Save as Draft or Submit), copy the exact message into 'Actual message', pick an Outcome, then restore the value before the next test. Rows added to tables save immediately, so delete test rows afterwards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After testing</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Send the filled sheet back; confirmed rules will be moved into 'Portal checks' with How found = Tested.</t>
         </is>
       </c>
     </row>
@@ -39253,4 +39322,1994 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Priority</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Area / PDF box</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Starting state</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Change to make</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expected result</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Known message</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actual message (fill in)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outcome (fill in)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restore after test</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Links (Portal checks / Rule register)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T00</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Setup</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whole return</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Return open, before any test</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Save a copy of the page as it is now: browser Print &gt; Save as PDF (whole page, all schedules), and list every table row. Never press Save as Draft or Submit during these tests.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reference copy for restoring values at the end.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keep the copy until the return is filed.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Setup</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: Designation</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As T00</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add ' TEST' to the end of the Declaration designation. Press Check and Calculate. Then press Back, reopen the return from Pending Tasks and look at the designation.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether Check and Calculate writes values into the stored draft. If ' TEST' is still there, every later test changes the draft until you restore it.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remove ' TEST' and press Check and Calculate.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T02</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Setup</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whole return</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No changes</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Press Check and Calculate.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baseline: the 10 known errors. Compare every later test with this list; only record messages that are new or that disappear.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See Portal checks P001-P010</t>
+        </is>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P001-P010</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section A and Section B together (Boxes 191 / 203, Box A)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section B in use</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enter 1 in Section A Box 11 (gifts) so that both Section A and Section B have figures.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page code says the server rejects a return with both sections filled. PDF only sets Box A to 0 (R015 defect).</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown: record exactly</t>
+        </is>
+      </c>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear Box 11.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R015</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T04</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: accounting period From / To</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period filled</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear both period dates.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error expected: period is needed to compute the tax-free bracket.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter both dates.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R012</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T05</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: accounting period From / To</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period filled</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Set To earlier than From (e.g. From 01/01/2025, To 31/12/2024).</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error expected; PDF does not check this.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original dates.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R012</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T06</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: accounting period</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period filled</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Set a period longer than 12 months, or one that does not end in tax year 2025.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error or warning expected (s.58 of the Regulation).</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original dates.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R012</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T07</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: residency status</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One residency box ticked</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untick all three residency boxes (Resident / Temporary resident / Non-resident).</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error expected; residency opens Box B, G, 88, 109-111.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-tick the original box.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R009-R011</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T08</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: Name</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name filled</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear the declarant's name.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error expected (same family as 'Please enter contact number').</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter the name.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T09</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: Designation</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filled</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear the designation.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error expected.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter the designation.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R027</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T10</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: Date</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filled or blank</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Clear the date. (b) Enter a date in the future. (c) Enter a date before the period end.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Error expected. (b)/(c) Unknown.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'The field A_DEC_DATE must be a date.' for invalid text</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record (a), (b), (c) separately</t>
+        </is>
+      </c>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original date.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R029, P032</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T11</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: Contact number</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blank (P010 fires)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Enter letters 'abc'. (b) Enter '+960 7771234'. (c) Enter '123'. (d) Enter a valid 7-digit number.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a)-(c) show whether a format check exists; (d) P010 should disappear.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'Please enter contact number' when blank</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record (a)-(d) separately</t>
+        </is>
+      </c>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear it again if it was blank in T00.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R028, P010</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T12</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">III Presentation currency vs II functional currency</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presentation blank (P005 fires)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Select Rufiyaa with II-b (e)-(h) showing USD. (b) Select USD with functional currency Rufiyaa.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF says: if functional currency is not MVR you must present in USD. Shows whether the portal blocks the mismatch.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'Please select the presentation currency' when blank</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record (a), (b)</t>
+        </is>
+      </c>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear both selections.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R038, R039, P005</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T13</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">II-a vs II-b functional currency</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">II-b blank (P003/P004 fire)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Tick an II-b option in (a)-(d) and (e)-(h). (b) Also tick an II-a option (first-year block).</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) P003/P004 should disappear. (b) Shows whether ticking both blocks is rejected (PDF allows it).</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See P003, P004</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record (a), (b)</t>
+        </is>
+      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untick everything you ticked.</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R035, R037, P003, P004</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T14</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IV Audit opinion</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opinion as filed</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Clear the audit opinion. (b) Select (e) 'Not required to audit'.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Error expected. (b) Shows whether 'Please upload audit report' (P008) and the directors' report error (P007) disappear.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record (a), (b)</t>
+        </is>
+      </c>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-select original opinion.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R040, P007, P008</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T15</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: Auditor registration number</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filled</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear the auditor registration number while opinion is (a)-(d).</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error expected; PDF does not check this.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter the number.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R013</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T16</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIII Bank accounts</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 rows (P006 fires)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add one bank row with all 4 fields. NOTE: rows save immediately. Then press Check and Calculate.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P006 should disappear. Confirms one row is enough.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See P006</t>
+        </is>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete the test row (Delete button on the row).</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R050, P006, P016</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T17</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">XIII Bank accounts row</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adding a row</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Try to save a bank row with Currency left as 'Select Currency'.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Row refused (client-side).</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Currency field is required.</t>
+        </is>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cancel the row.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P016</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T18</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section B: amount boxes</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Figures as filed</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enter a negative figure in a manual Section B income box (e.g. the turnover / revenue box).</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether negatives are blocked on income boxes.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original figure.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T19</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computation: Box B foreign tax credit</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resident</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enter a Box B figure greater than Box A.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: no cap (C can go negative). Shows whether the portal caps it.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original (usually 0).</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R016, R017</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T20</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computation: Box N amount being paid</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enter a Box N figure different from Box M.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: not compared. Shows whether the portal warns.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original.</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R024</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T21</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box 31-33 / 159-161 allocation (Note 1)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If the box is typeable, enter more than the box it is capped by (e.g. Box 159 &gt; Box 156).</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note 1 says it must not exceed; shows whether the portal blocks or recalculates.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original.</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note 1 rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T22</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box 192 tax brackets (Note 5)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If brackets are typeable, put more into the 0% bracket than its size.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note 5: amounts must not exceed the bracket size.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original.</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note 4/5 rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T23</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Group companies count (A) vs X Group companies table</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Enter a count of 2 with no rows in table X. (b) Add 1 row but leave count 0. (Rows save immediately.)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether the count must match the table.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record (a), (b)</t>
+        </is>
+      </c>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restore count; delete any test row.</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R008, R047, P019</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T24</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VII Thin capitalisation</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Untick all (a)-(d). (b) Tick two of them.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether the item is required or single-choice.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record (a), (b)</t>
+        </is>
+      </c>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restore original ticks.</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R044</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T25</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIII Section 11(r) only? / IX Special return s.48</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Answered</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear the Yes/No answer on VIII, then on IX (one at a time).</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error expected if mandatory.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record VIII, IX</t>
+        </is>
+      </c>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-select original answers.</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R045, R046</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T26</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I Basis of accounts</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accrual/Cash ticked</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untick both.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Error expected.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-tick original.</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R034</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T27</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document checklist ticks</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untick all checklist boxes (financial statements, notes, audit, etc.).</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether ticks are checked separately from uploads (P007-P009).</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-tick original boxes.</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R032</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T28</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 item 3A</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 showing</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear both item 3A boxes, press Check and Calculate.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Browser alert, boxes outlined red, nothing sent to server.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item no 3A cannot be left blank; if there is no sale/purchase to report, then enter 0.</t>
+        </is>
+      </c>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original (or 0).</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P011</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T29</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 item 4.3(a) / (b)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Errors P001/P002 fire</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tick 'did not receive any loans from associates' and 'did not give any loans to associates'.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P001 and P002 should disappear.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See P001, P002</t>
+        </is>
+      </c>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untick both.</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P001, P002</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T30</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 conditions block</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(a) Untick all conditions and the 'not required' box. (b) Tick 'not required' and a condition together.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether one choice is mandatory and whether the combination is rejected.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record (a), (b)</t>
+        </is>
+      </c>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restore original ticks.</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T31</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 part 1 shareholders</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Note the total of shareholding %. If you can, add a test row so the total exceeds 100%.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether the total is checked (rows save immediately).</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete the test row.</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P023</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T32</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supporting documents</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None uploaded (P007-P009 fire)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only if you have the real documents ready: upload the auditor's report only.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P008 should disappear; P007 and P009 remain. Also note whether the 'I declare that the Auditor's Report...' tick becomes required.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See P007-P009</t>
+        </is>
+      </c>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keep (they are needed anyway) or delete the upload.</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P007-P009</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T33</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statement of donations row</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adding a row</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add a donation dated outside 2025, then press Check and Calculate.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether the date must fall in the tax year (not checked client-side).</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete the test row.</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R177, P021</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T34</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Statement of donations: Box 27 / 155</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Donations as filed</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type a figure directly into Box 27 or Box 155.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box resets to 0 and the donations table opens.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This value will be auto populated from statement of donations table. Please scroll down and fill the statement of donations table.</t>
+        </is>
+      </c>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None needed.</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P015</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T35</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sponsorship statements (teams / media)</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adding a row</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add a sponsorship paid outside 2025, then press Check and Calculate.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printed note: payment date must fall in the tax year. Shows whether it is enforced.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete the test row.</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P022</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T36</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Numeric boxes generally</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As filed</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type 'abc' into any amount box and click away.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Client-side format message.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The field &lt;box&gt; must be a number.</t>
+        </is>
+      </c>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-enter original.</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P031</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T37</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 6 items 8-13</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 6 not used</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tick one item 8 box (e.g. 8.8 options) and leave item 11 empty.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows whether the opened items become mandatory.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown</t>
+        </is>
+      </c>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Untick; items 9-13 clear automatically.</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P030</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I39">
+      <formula1>"As expected,Different message,No error,New error,Not run"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Record first MIRAconnect test results in MIRA 604 register
Portal checks P033-P044: basis of accounts, audit opinion, items VIII
and IX and a numeric contact number are mandatory; Section A and
Section B cannot both be filled; accounting period, residency, auditor
number and industry code are not required; upload errors follow the
checklist / audit opinion; Check and Calculate does not save values.
Test script columns H-I filled for the tests run; the rest marked
Not run. Read me gains a status line and a one-line summary.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mira-604/MIRA_604_v26.1_validation_register.xlsx
+++ b/mira-604/MIRA_604_v26.1_validation_register.xlsx
@@ -266,8 +266,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PortalChecks" displayName="PortalChecks" ref="A1:J33" headerRowCount="1">
-  <autoFilter ref="A1:J33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PortalChecks" displayName="PortalChecks" ref="A1:J45" headerRowCount="1">
+  <autoFilter ref="A1:J45"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Portal screen/step"/>
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -957,6 +957,30 @@
       <c r="B35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Send the filled sheet back; confirmed rules will be moved into 'Portal checks' with How found = Tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status 20 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run so far: baseline (T02), T01, T03, T04, T07, T11a/d, T14a, T15, T25, T26, T27 (batch A: several changes in one Check). Results are in 'Portal checks' P033-P044 and in the test script columns H-I. Not yet run: T05, T06, T12, T13, T16-T24, T28-T37, and the single-change reruns of T14b and T27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal findings in one line</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mandatory in the portal but not in the PDF: II-b, III, I basis, IV audit opinion, VIII, IX, XIII bank account, contact number (numeric), uploads (driven by checklist/opinion), Schedule 4 items 3A and 4.3. NOT required by either: accounting period, residency, auditor number, industry code. Section A and Section B cannot both be filled.</t>
         </is>
       </c>
     </row>
@@ -37585,7 +37609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -39313,6 +39337,630 @@
       <c r="J33" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PDF uses DDMMYYYY comb cells; neither checks To is after From (client side).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I Basis of accounts</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I Basis of accounts</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single choice: Accrual / Cash</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please select the basis your accounts are prepared on</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R034</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: radio, not checked. Portal: mandatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IV Audit opinion</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IV Audit opinion</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single choice (a)-(e)</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please select the type of audit opinion</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R040</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: radio, not checked. Portal: mandatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIII Non-resident shipping/aircraft, s.11(r) income only?</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIII Section 11(r) only?</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes / No</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You must provide an answer to item VIII on page 2</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R045</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: not checked. Portal: mandatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IX Special return under s.48</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IX Special return s48</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes / No</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You must provide an answer to item IX on page 2</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R046</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: not checked, no downstream effect. Portal: mandatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: contact number format</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declaration: Contact Number</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes; digits only</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Numeric only; no length or leading-digit check seen (0000000 accepted)</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please enter contact number. Contact number must have numeric numbers only</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A: 'abc' rejected; 0000000 accepted)</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R028</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: numeric whole number, not required. Portal: required and numeric.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section A and Section B / Schedule 1 both completed</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section A Boxes 1-52 vs Schedule 1 and Section B</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule: a return cannot carry figures in Section A and in Schedule 1 / Section B at the same time</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entering 1 in Box 11 on a Section B return triggers it</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You cannot fill in Schedule One if you are completing Section A</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R015</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF only sets Box A to 0 when both 191 and 203 are filled. Portal blocks the return.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: accounting period From / To</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header accounting period</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No: both dates blank gave no error</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date format only (client side)</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R012, P032</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Neither PDF nor portal requires the period. Reversed / over-12-month periods not yet tested (T05, T06).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: residency status</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header residency status</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No: no residency ticked gave no error</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Three exclusive ticks (client side)</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R009</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Neither PDF nor portal requires residency, although it drives Boxes B, G, 88, 109-111.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: auditor registration number</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header Auditor Registration Number</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No: blank gave no error (audit opinion was also blank in the same run)</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dropdown of registered auditors</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R013</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not required even though it is a dropdown. Retest with an audit opinion (a)-(d) selected (T15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: industry code</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header Industry Code</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No: blank in the baseline run and never flagged</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dropdown</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (baseline, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header Industry Code</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not required in either.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supporting document uploads: what triggers P007-P009</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document checklist; IV Audit opinion</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: all three upload errors disappeared when the document checklist was unticked AND the audit opinion was cleared in the same run</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upload requirement follows the checklist ticks and/or the audit opinion</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(P007-P009 no longer shown)</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch A, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R032, R040</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which of the two drives it is not yet separated (T14b, T27 to be run one at a time).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whole return: does Check and Calculate save?</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule: Check and Calculate validates the posted values but does NOT write them to the stored draft; reopening the return shows the last saved values. Table rows (bank accounts, owners, Schedule 4 etc.) save immediately on Add/Delete.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (T01, 20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only Save as Draft / Submit persist box values.</t>
         </is>
       </c>
     </row>
@@ -39439,8 +40087,16 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Snapshot of every field and table row taken 20 Oct 2026 (kept outside the repo).</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Keep the copy until the return is filed.</t>
@@ -39488,8 +40144,16 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contact number set to 0000000, Check and Calculate pressed, return reopened from the server: field was blank again. Check and Calculate does not save box values.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done: not persisted</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Remove ' TEST' and press Check and Calculate.</t>
@@ -39537,8 +40201,16 @@
           <t xml:space="preserve">See Portal checks P001-P010</t>
         </is>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10 errors, exactly P001-P010.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As expected</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -39586,8 +40258,16 @@
           <t xml:space="preserve">Unknown: record exactly</t>
         </is>
       </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You cannot fill in Schedule One if you are completing Section A</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New error</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Clear Box 11.</t>
@@ -39635,8 +40315,16 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No message for blank From / To.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No error</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter both dates.</t>
@@ -39685,7 +40373,11 @@
         </is>
       </c>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original dates.</t>
@@ -39734,7 +40426,11 @@
         </is>
       </c>
       <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original dates.</t>
@@ -39782,8 +40478,16 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No message with no residency ticked.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No error</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-tick the original box.</t>
@@ -39831,8 +40535,16 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cannot run: declarant name is a hidden, pre-filled field on the portal.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not applicable</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter the name.</t>
@@ -39880,8 +40592,16 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cannot run: designation is a hidden, pre-filled field on the portal.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not applicable</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter the designation.</t>
@@ -39934,7 +40654,11 @@
           <t xml:space="preserve">Record (a), (b), (c) separately</t>
         </is>
       </c>
-      <c r="I12" s="2"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not applicable</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original date.</t>
@@ -39987,7 +40711,11 @@
           <t xml:space="preserve">Record (a)-(d) separately</t>
         </is>
       </c>
-      <c r="I13" s="2"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New error</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Clear it again if it was blank in T00.</t>
@@ -40040,7 +40768,11 @@
           <t xml:space="preserve">Record (a), (b)</t>
         </is>
       </c>
-      <c r="I14" s="2"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Clear both selections.</t>
@@ -40093,7 +40825,11 @@
           <t xml:space="preserve">Record (a), (b)</t>
         </is>
       </c>
-      <c r="I15" s="2"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Untick everything you ticked.</t>
@@ -40146,7 +40882,11 @@
           <t xml:space="preserve">Record (a), (b)</t>
         </is>
       </c>
-      <c r="I16" s="2"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New error</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-select original opinion.</t>
@@ -40194,8 +40934,16 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No message with the auditor number blank (audit opinion was blank in the same run; retest with opinion (a)-(d)).</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No error</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter the number.</t>
@@ -40244,7 +40992,11 @@
         </is>
       </c>
       <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Delete the test row (Delete button on the row).</t>
@@ -40293,7 +41045,11 @@
         </is>
       </c>
       <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Cancel the row.</t>
@@ -40342,7 +41098,11 @@
         </is>
       </c>
       <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original figure.</t>
@@ -40391,7 +41151,11 @@
         </is>
       </c>
       <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original (usually 0).</t>
@@ -40440,7 +41204,11 @@
         </is>
       </c>
       <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original.</t>
@@ -40489,7 +41257,11 @@
         </is>
       </c>
       <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original.</t>
@@ -40538,7 +41310,11 @@
         </is>
       </c>
       <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original.</t>
@@ -40591,7 +41367,11 @@
           <t xml:space="preserve">Record (a), (b)</t>
         </is>
       </c>
-      <c r="I25" s="2"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Restore count; delete any test row.</t>
@@ -40644,7 +41424,11 @@
           <t xml:space="preserve">Record (a), (b)</t>
         </is>
       </c>
-      <c r="I26" s="2"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Restore original ticks.</t>
@@ -40697,7 +41481,11 @@
           <t xml:space="preserve">Record VIII, IX</t>
         </is>
       </c>
-      <c r="I27" s="2"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New error</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-select original answers.</t>
@@ -40745,8 +41533,16 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please select the basis your accounts are prepared on</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New error</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-tick original.</t>
@@ -40794,8 +41590,16 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All checklist ticks off (with audit opinion also blank): the three upload errors P007-P009 disappeared. Rerun alone to confirm the checklist is the trigger.</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Different message</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-tick original boxes.</t>
@@ -40844,7 +41648,11 @@
         </is>
       </c>
       <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original (or 0).</t>
@@ -40893,7 +41701,11 @@
         </is>
       </c>
       <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Untick both.</t>
@@ -40946,7 +41758,11 @@
           <t xml:space="preserve">Record (a), (b)</t>
         </is>
       </c>
-      <c r="I32" s="2"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Restore original ticks.</t>
@@ -40995,7 +41811,11 @@
         </is>
       </c>
       <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Delete the test row.</t>
@@ -41044,7 +41864,11 @@
         </is>
       </c>
       <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Keep (they are needed anyway) or delete the upload.</t>
@@ -41093,7 +41917,11 @@
         </is>
       </c>
       <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Delete the test row.</t>
@@ -41142,7 +41970,11 @@
         </is>
       </c>
       <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">None needed.</t>
@@ -41191,7 +42023,11 @@
         </is>
       </c>
       <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Delete the test row.</t>
@@ -41240,7 +42076,11 @@
         </is>
       </c>
       <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Re-enter original.</t>
@@ -41289,7 +42129,11 @@
         </is>
       </c>
       <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Untick; items 9-13 clear automatically.</t>

</xml_diff>

<commit_message>
Record MIRAconnect test batches B and C in MIRA 604 register
Portal checks P045-P056: group count must match table X and cannot
be 0; Box B needs uploads and cannot exceed Box A; Boxes C and E
cannot be negative; a Schedule 4 condition must be ticked; audit
opinion (e) is rejected when revenue requires an audit; period order,
negative income boxes, Box N vs M, presentation vs functional
currency and thin-cap ticks are not checked. Test script outcomes
updated; Read me notes the stop and what remains untested.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mira-604/MIRA_604_v26.1_validation_register.xlsx
+++ b/mira-604/MIRA_604_v26.1_validation_register.xlsx
@@ -266,8 +266,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PortalChecks" displayName="PortalChecks" ref="A1:J45" headerRowCount="1">
-  <autoFilter ref="A1:J45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PortalChecks" displayName="PortalChecks" ref="A1:J57" headerRowCount="1">
+  <autoFilter ref="A1:J57"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Portal screen/step"/>
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -981,6 +981,30 @@
       <c r="B37" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mandatory in the portal but not in the PDF: II-b, III, I basis, IV audit opinion, VIII, IX, XIII bank account, contact number (numeric), uploads (driven by checklist/opinion), Schedule 4 items 3A and 4.3. NOT required by either: accounting period, residency, auditor number, industry code. Section A and Section B cannot both be filled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Batches B and C (20 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Also run: T05, T12a, T13, T14b, T18, T19, T20, T23a, T24, T29, T30a. Results in Portal checks P045-P056. Testing stopped at the user's request; the return was reloaded from the server with no values saved. Still not run: T06, T16, T17, T21, T22, T28, T31-T37, T23b, T30b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Portal-only rules found in B and C</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Group count must match table X and cannot be 0; Box B needs uploads and cannot exceed Box A; Boxes C and E cannot be negative; a Schedule 4 condition (or not-required) must be ticked; audit opinion (e) is rejected when revenue requires an audit. NOT checked by the portal: period order, negative income boxes, Box N vs M, presentation vs functional currency, thin-cap ticks.</t>
         </is>
       </c>
     </row>
@@ -37609,7 +37633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -39961,6 +39985,630 @@
       <c r="J45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Only Save as Draft / Submit persist box values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header group count vs X Group companies table</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: Group companies count; X Group companies</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: if a group count is entered, table X must have that many rows</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Count must equal the number of rows in X</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please enter all the details required in item X on page 3 / Number of companies that share the tax free bracket in item X must match the number declared on page 1 as the number of companies in the group that are liable to income tax in Maldives</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch B: count 2, 0 rows)</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R008, R047</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: no link between the count and the table. Portal: both messages fire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header group count = 0</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header: Group companies count</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule: 0 or negative is rejected; leave blank if not in a group</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positive whole number or blank</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number of companies in the Group cannot be zero or negative. Please leave it blank if not applicable.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch C: count 0)</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R008</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF accepts 0 (used as A in Note 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box B foreign tax credit: supporting documents</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computation Box B</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: Box B &gt; 0 requires an upload</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upload under supporting documents</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please upload the supporting documents in order to claim foreign tax credit in Box B on page 1</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch B: Box B 999,999)</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R016</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: printed note 'attach explanations' only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box B vs Box A</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computation Boxes A, B</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule: Box B must not exceed Box A</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cap</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box B should not be greater than Box A</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch B)</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R016, R017</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: no cap, Box C goes negative. Portal blocks it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Boxes C and E negative</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computation Boxes C, E</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule: C and E must not be negative</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Floor at 0</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box C and E should not be negative</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch B: C recalculated to -990,472.72)</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R017</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: no floor. Portal blocks the return.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 conditions block (bullet one)</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes: at least one condition, or the 'not required' box, must be ticked</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tick boxes</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please tick the applicable boxes under Bullet one on Page I of Schedule 4 to indicate which conditions apply to you / Please tick the applicable boxes under Bullet one on Page I of Schedule 4</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch C: all unticked)</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two messages fire together. With no condition ticked the 4.3(a)/(b) errors are not raised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IV Audit opinion (e) 'Not required to audit' vs revenue</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IV Audit opinion</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: (e) is rejected when revenue is above the audit threshold; the three upload errors stay</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server compares revenue with the audit threshold</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are required to audit based on your revenue</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch C)</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R040, P007-P009</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF: no link to revenue. Portal enforces the audit requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accounting period To before From</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header accounting period</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No: To = 31/12/2024 with From = 01/01/2025 gave no error</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not checked</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch C)</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R012, P039</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Neither PDF nor portal checks the order of the dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VII Thin capitalisation ticks</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VII Thin capitalization</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No: none ticked (baseline) and two ticked (batch B) both passed</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Independent tick boxes</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (baseline, batch B)</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R044</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same as PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negative income box; Box N vs Box M</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section B Box 151; Computation Box N</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No: Box 151 = -5 and Box N (1.00) different from Box M both passed</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not checked</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch B)</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R024</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same as PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">III presentation currency vs II functional currency; II-a with II-b</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">III Presentation currency; II-a / II-b</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No: Rufiyaa presentation with USD functional currency passed; II-a and II-b ticked together passed</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not checked</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(none)</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch C)</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R035, R037, R039</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The printed rule 'must present in USD' is not enforced in either.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check and Calculate (server)</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule 4 item 4.3 no-loans ticks</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not in PDF v26.1</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conditional: ticking 'did not receive / give any loans' clears the 4.3(a)/(b) errors</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tick boxes</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(P001, P002 no longer shown)</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tested (batch B)</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P001, P002</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirms the two ways to satisfy item 4.3.</t>
         </is>
       </c>
     </row>
@@ -40372,10 +41020,14 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No message with To (31/12/2024) before From (01/01/2025).</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">No error</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -40765,12 +41417,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record (a), (b)</t>
+          <t xml:space="preserve">(a) Rufiyaa presentation with USD functional currency: no message.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">No error</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -40822,12 +41474,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record (a), (b)</t>
+          <t xml:space="preserve">(a) P003/P004 cleared. (b) II-a and II-b ticked together: no message.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">No error</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -40879,7 +41531,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record (a), (b)</t>
+          <t xml:space="preserve">(a) blank: "Please select the type of audit opinion". (b) (e) Not required: "You are required to audit based on your revenue"; upload errors P007-P009 remain.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -41097,10 +41749,14 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H20" s="2"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box 151 = -5: no message.</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">No error</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -41150,10 +41806,14 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box B 999,999 &gt; Box A: "Box B should not be greater than Box A", "Box C and E should not be negative", "Please upload the supporting documents in order to claim foreign tax credit in Box B on page 1".</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">New error</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -41203,10 +41863,14 @@
           <t xml:space="preserve">Unknown</t>
         </is>
       </c>
-      <c r="H22" s="2"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box N = 1.00 with Box M different: no message.</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">No error</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -41364,12 +42028,12 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record (a), (b)</t>
+          <t xml:space="preserve">(a) count 2, no rows: "Please enter all the details required in item X on page 3" and "Number of companies that share the tax free bracket in item X must match the number declared on page 1...". Count 0: "Number of companies in the Group cannot be zero or negative. Please leave it blank if not applicable." (b) not run.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">New error</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -41421,12 +42085,12 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record (a), (b)</t>
+          <t xml:space="preserve">(a) none ticked (baseline): no message. (b) A and B ticked: no message.</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">No error</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -41700,10 +42364,14 @@
           <t xml:space="preserve">See P001, P002</t>
         </is>
       </c>
-      <c r="H31" s="2"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Both no-loans ticks: P001 and P002 cleared.</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">As expected</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -41755,12 +42423,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record (a), (b)</t>
+          <t xml:space="preserve">(a) all unticked: "Please tick the applicable boxes under Bullet one on Page I of Schedule 4 to indicate which conditions apply to you" and "Please tick the applicable boxes under Bullet one on Page I of Schedule 4". 4.3 errors not raised in this state. (b) not run.</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not run</t>
+          <t xml:space="preserve">New error</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">

</xml_diff>